<commit_message>
Added evals on all the Naive RAG Fields
</commit_message>
<xml_diff>
--- a/Records.xlsx
+++ b/Records.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Projects\rag-dissertation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D44ED7E-080D-4918-A927-80A5CCB8F680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92D6711E-328A-4293-A458-F864C65F895A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{F211E78F-65A6-4528-B59A-5C2BEDBB7ED5}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="101">
   <si>
     <t>LITERATURE REVIEW</t>
   </si>
@@ -332,6 +332,12 @@
   </si>
   <si>
     <t>Climate</t>
+  </si>
+  <si>
+    <t>Science</t>
+  </si>
+  <si>
+    <t>General</t>
   </si>
 </sst>
 </file>
@@ -663,20 +669,20 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1603,7 +1609,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C0FA7FA-43F7-4BFF-A8EE-58A2C3A96766}">
-  <dimension ref="G3:O14"/>
+  <dimension ref="G3:O16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="23.42578125" customWidth="1"/>
@@ -1625,25 +1631,25 @@
       <c r="G8" s="45" t="s">
         <v>80</v>
       </c>
-      <c r="H8" s="46" t="s">
+      <c r="H8" s="51" t="s">
         <v>90</v>
       </c>
-      <c r="I8" s="46"/>
-      <c r="J8" s="47" t="s">
+      <c r="I8" s="51"/>
+      <c r="J8" s="48" t="s">
         <v>86</v>
       </c>
-      <c r="K8" s="47"/>
-      <c r="L8" s="47"/>
-      <c r="M8" s="47"/>
-      <c r="N8" s="47"/>
-      <c r="O8" s="47"/>
+      <c r="K8" s="48"/>
+      <c r="L8" s="48"/>
+      <c r="M8" s="48"/>
+      <c r="N8" s="48"/>
+      <c r="O8" s="48"/>
     </row>
     <row r="9" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G9" s="48"/>
-      <c r="H9" s="51" t="s">
+      <c r="G9" s="46"/>
+      <c r="H9" s="47" t="s">
         <v>81</v>
       </c>
-      <c r="I9" s="51" t="s">
+      <c r="I9" s="47" t="s">
         <v>89</v>
       </c>
       <c r="J9" s="49" t="s">
@@ -1658,9 +1664,9 @@
       <c r="O9" s="50"/>
     </row>
     <row r="10" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G10" s="48"/>
-      <c r="H10" s="48"/>
-      <c r="I10" s="48"/>
+      <c r="G10" s="46"/>
+      <c r="H10" s="46"/>
+      <c r="I10" s="46"/>
       <c r="J10" s="45" t="s">
         <v>82</v>
       </c>
@@ -1713,6 +1719,16 @@
       </c>
       <c r="I14" t="s">
         <v>98</v>
+      </c>
+    </row>
+    <row r="15" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="I15" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="16" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="I16" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Experiment 1 - Naive RAG Fully complete
</commit_message>
<xml_diff>
--- a/Records.xlsx
+++ b/Records.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Projects\rag-dissertation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92D6711E-328A-4293-A458-F864C65F895A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9D99684-2C03-4492-B3BD-4A925AA9F676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{F211E78F-65A6-4528-B59A-5C2BEDBB7ED5}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="116">
   <si>
     <t>LITERATURE REVIEW</t>
   </si>
@@ -286,9 +286,6 @@
     <t>HM</t>
   </si>
   <si>
-    <t>FM</t>
-  </si>
-  <si>
     <t>AR</t>
   </si>
   <si>
@@ -298,9 +295,6 @@
     <t>Evaluation</t>
   </si>
   <si>
-    <t>Baseline</t>
-  </si>
-  <si>
     <t>Post Retrieval</t>
   </si>
   <si>
@@ -328,23 +322,74 @@
     <t>Corporate</t>
   </si>
   <si>
-    <t>IPCC</t>
-  </si>
-  <si>
-    <t>Climate</t>
-  </si>
-  <si>
     <t>Science</t>
   </si>
   <si>
     <t>General</t>
+  </si>
+  <si>
+    <t>Pre Retrieval - Baseline</t>
+  </si>
+  <si>
+    <t>FF</t>
+  </si>
+  <si>
+    <t>Constants</t>
+  </si>
+  <si>
+    <t>Embeddings Model</t>
+  </si>
+  <si>
+    <t>Generator Model</t>
+  </si>
+  <si>
+    <t>Judge Model</t>
+  </si>
+  <si>
+    <t>Question Type</t>
+  </si>
+  <si>
+    <t>Chunk Size</t>
+  </si>
+  <si>
+    <t>Chunk Overlap</t>
+  </si>
+  <si>
+    <t>Hugging Face Embeddings: sentence-transformers/all-mpnet-base-v2</t>
+  </si>
+  <si>
+    <t>Qwen 3.5:2b</t>
+  </si>
+  <si>
+    <t>Gemma4:e4b</t>
+  </si>
+  <si>
+    <t>Factual</t>
+  </si>
+  <si>
+    <t>&gt;=0.5</t>
+  </si>
+  <si>
+    <t>Eval Threshold Metric</t>
+  </si>
+  <si>
+    <t>UNEP Dataset</t>
+  </si>
+  <si>
+    <t>IPCC Dataset</t>
+  </si>
+  <si>
+    <t>20 News Group Dataset</t>
+  </si>
+  <si>
+    <t>Environment</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -447,6 +492,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -510,7 +561,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -533,12 +584,90 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color theme="9"/>
+      </left>
+      <right style="thick">
+        <color theme="9"/>
+      </right>
+      <top style="thick">
+        <color theme="9"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color theme="9"/>
+      </left>
+      <right style="thick">
+        <color theme="9"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color theme="9"/>
+      </left>
+      <right style="thick">
+        <color theme="9"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color theme="9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -673,6 +802,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -684,6 +816,29 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1609,134 +1764,330 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C0FA7FA-43F7-4BFF-A8EE-58A2C3A96766}">
-  <dimension ref="G3:O16"/>
+  <dimension ref="C3:L38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="7" max="7" width="23.42578125" customWidth="1"/>
-    <col min="8" max="8" width="20.85546875" customWidth="1"/>
-    <col min="9" max="9" width="19.28515625" customWidth="1"/>
-    <col min="10" max="10" width="16.28515625" customWidth="1"/>
-    <col min="11" max="11" width="19.85546875" customWidth="1"/>
+    <col min="3" max="3" width="16.5703125" customWidth="1"/>
+    <col min="4" max="4" width="27.85546875" customWidth="1"/>
+    <col min="5" max="5" width="24.7109375" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" customWidth="1"/>
+    <col min="11" max="11" width="14.140625" customWidth="1"/>
     <col min="12" max="12" width="17.85546875" customWidth="1"/>
     <col min="13" max="13" width="17" customWidth="1"/>
     <col min="14" max="14" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="4:9" x14ac:dyDescent="0.25">
       <c r="I3" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="8" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G8" s="45" t="s">
+    <row r="9" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D9" s="53" t="s">
+        <v>99</v>
+      </c>
+      <c r="E9" s="53"/>
+    </row>
+    <row r="10" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D10" s="44" t="s">
+        <v>104</v>
+      </c>
+      <c r="E10" s="44">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="11" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D11" s="44" t="s">
+        <v>105</v>
+      </c>
+      <c r="E11" s="44">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D12" s="44" t="s">
+        <v>100</v>
+      </c>
+      <c r="E12" s="48" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="13" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D13" s="44" t="s">
+        <v>101</v>
+      </c>
+      <c r="E13" s="44" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="14" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D14" s="44" t="s">
+        <v>102</v>
+      </c>
+      <c r="E14" s="44" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="15" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D15" s="44" t="s">
+        <v>103</v>
+      </c>
+      <c r="E15" s="44" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="16" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D16" s="44" t="s">
+        <v>111</v>
+      </c>
+      <c r="E16" s="44" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="20" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C20" s="45" t="s">
         <v>80</v>
       </c>
-      <c r="H8" s="51" t="s">
+      <c r="D20" s="52" t="s">
+        <v>88</v>
+      </c>
+      <c r="E20" s="52"/>
+      <c r="F20" s="49" t="s">
+        <v>85</v>
+      </c>
+      <c r="G20" s="49"/>
+      <c r="H20" s="49"/>
+      <c r="I20" s="49"/>
+      <c r="J20" s="49"/>
+      <c r="K20" s="49"/>
+    </row>
+    <row r="21" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C21" s="46"/>
+      <c r="D21" s="47" t="s">
+        <v>87</v>
+      </c>
+      <c r="E21" s="47" t="s">
+        <v>81</v>
+      </c>
+      <c r="F21" s="56" t="s">
+        <v>97</v>
+      </c>
+      <c r="G21" s="50"/>
+      <c r="H21" s="50"/>
+      <c r="I21" s="61" t="s">
+        <v>86</v>
+      </c>
+      <c r="J21" s="51"/>
+      <c r="K21" s="51"/>
+    </row>
+    <row r="22" spans="3:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="C22" s="46"/>
+      <c r="D22" s="46"/>
+      <c r="E22" s="54"/>
+      <c r="F22" s="57" t="s">
+        <v>82</v>
+      </c>
+      <c r="G22" s="55" t="s">
+        <v>83</v>
+      </c>
+      <c r="H22" s="60" t="s">
+        <v>98</v>
+      </c>
+      <c r="I22" s="57" t="s">
+        <v>82</v>
+      </c>
+      <c r="J22" s="55" t="s">
+        <v>83</v>
+      </c>
+      <c r="K22" s="45" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="23" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="D23" s="44" t="s">
         <v>90</v>
       </c>
-      <c r="I8" s="51"/>
-      <c r="J8" s="48" t="s">
-        <v>86</v>
-      </c>
-      <c r="K8" s="48"/>
-      <c r="L8" s="48"/>
-      <c r="M8" s="48"/>
-      <c r="N8" s="48"/>
-      <c r="O8" s="48"/>
-    </row>
-    <row r="9" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G9" s="46"/>
-      <c r="H9" s="47" t="s">
-        <v>81</v>
-      </c>
-      <c r="I9" s="47" t="s">
+      <c r="E23" s="44" t="s">
         <v>89</v>
       </c>
-      <c r="J9" s="49" t="s">
-        <v>87</v>
-      </c>
-      <c r="K9" s="49"/>
-      <c r="L9" s="49"/>
-      <c r="M9" s="50" t="s">
-        <v>88</v>
-      </c>
-      <c r="N9" s="50"/>
-      <c r="O9" s="50"/>
-    </row>
-    <row r="10" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G10" s="46"/>
-      <c r="H10" s="46"/>
-      <c r="I10" s="46"/>
-      <c r="J10" s="45" t="s">
-        <v>82</v>
-      </c>
-      <c r="K10" s="45" t="s">
-        <v>83</v>
-      </c>
-      <c r="L10" s="45" t="s">
+      <c r="F23" s="58">
+        <v>0</v>
+      </c>
+      <c r="G23" s="44">
+        <v>1</v>
+      </c>
+      <c r="H23" s="44">
+        <v>0</v>
+      </c>
+      <c r="I23" s="58">
+        <v>1</v>
+      </c>
+      <c r="J23" s="44">
+        <v>1</v>
+      </c>
+      <c r="K23" s="44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="D24" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="E24" s="44" t="s">
+        <v>91</v>
+      </c>
+      <c r="F24" s="58">
+        <v>0</v>
+      </c>
+      <c r="G24" s="44">
+        <v>1</v>
+      </c>
+      <c r="H24" s="44">
+        <v>1</v>
+      </c>
+      <c r="I24" s="58">
+        <v>1</v>
+      </c>
+      <c r="J24" s="44">
+        <v>1</v>
+      </c>
+      <c r="K24" s="44">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="25" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C25" s="44" t="s">
         <v>84</v>
       </c>
-      <c r="M10" s="45" t="s">
-        <v>82</v>
-      </c>
-      <c r="N10" s="45" t="s">
-        <v>83</v>
-      </c>
-      <c r="O10" s="45" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="11" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="H11" t="s">
-        <v>91</v>
-      </c>
-      <c r="I11" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="12" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="H12" t="s">
+      <c r="D25" s="44" t="s">
+        <v>94</v>
+      </c>
+      <c r="E25" s="44" t="s">
         <v>93</v>
       </c>
-      <c r="I12" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="13" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G13" s="44" t="s">
-        <v>85</v>
-      </c>
-      <c r="H13" t="s">
+      <c r="F25" s="58">
+        <v>0</v>
+      </c>
+      <c r="G25" s="44">
+        <v>0.75</v>
+      </c>
+      <c r="H25" s="44">
+        <v>0</v>
+      </c>
+      <c r="I25" s="58">
+        <v>1</v>
+      </c>
+      <c r="J25" s="44">
+        <v>1</v>
+      </c>
+      <c r="K25" s="44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="D26" s="44" t="s">
+        <v>115</v>
+      </c>
+      <c r="E26" s="44" t="s">
+        <v>113</v>
+      </c>
+      <c r="F26" s="58">
+        <v>0</v>
+      </c>
+      <c r="G26" s="44">
+        <v>0.84599999999999997</v>
+      </c>
+      <c r="H26" s="44">
+        <v>1</v>
+      </c>
+      <c r="I26" s="58">
+        <v>1</v>
+      </c>
+      <c r="J26" s="44">
+        <v>1</v>
+      </c>
+      <c r="K26" s="44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="D27" s="44" t="s">
         <v>95</v>
       </c>
-      <c r="I13" t="s">
+      <c r="E27" s="44" t="s">
+        <v>112</v>
+      </c>
+      <c r="F27" s="58">
+        <v>1</v>
+      </c>
+      <c r="G27" s="44">
+        <v>1</v>
+      </c>
+      <c r="H27" s="44">
+        <v>1</v>
+      </c>
+      <c r="I27" s="58">
+        <v>0</v>
+      </c>
+      <c r="J27" s="44">
+        <v>1</v>
+      </c>
+      <c r="K27" s="44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="D28" s="44" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="14" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="H14" t="s">
-        <v>97</v>
-      </c>
-      <c r="I14" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="15" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="I15" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="16" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="I16" t="s">
-        <v>100</v>
-      </c>
+      <c r="E28" s="44" t="s">
+        <v>114</v>
+      </c>
+      <c r="F28" s="58">
+        <v>0</v>
+      </c>
+      <c r="G28" s="44">
+        <v>0.8</v>
+      </c>
+      <c r="H28" s="44">
+        <v>0</v>
+      </c>
+      <c r="I28" s="58">
+        <v>0</v>
+      </c>
+      <c r="J28" s="44">
+        <v>0.5</v>
+      </c>
+      <c r="K28" s="44">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="29" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E29" s="44"/>
+      <c r="F29" s="59"/>
+      <c r="I29" s="59"/>
+    </row>
+    <row r="30" spans="3:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="36" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L36" s="44"/>
+    </row>
+    <row r="37" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L37" s="44"/>
+    </row>
+    <row r="38" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L38" s="44"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="J8:O8"/>
-    <mergeCell ref="J9:L9"/>
-    <mergeCell ref="M9:O9"/>
-    <mergeCell ref="H8:I8"/>
+  <mergeCells count="5">
+    <mergeCell ref="F20:K20"/>
+    <mergeCell ref="F21:H21"/>
+    <mergeCell ref="I21:K21"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D9:E9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added Results to excel file & working on ocotber presentation
</commit_message>
<xml_diff>
--- a/Records.xlsx
+++ b/Records.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Projects\rag-dissertation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9D99684-2C03-4492-B3BD-4A925AA9F676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0E3FD74-BA31-4EA2-9074-2AE5C73790FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{F211E78F-65A6-4528-B59A-5C2BEDBB7ED5}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="127">
   <si>
     <t>LITERATURE REVIEW</t>
   </si>
@@ -274,9 +274,6 @@
     <t>Survey compares different RAGs against Accuracy vs Efficiency across various fields</t>
   </si>
   <si>
-    <t>Results/Outcomes</t>
-  </si>
-  <si>
     <t>Architecture</t>
   </si>
   <si>
@@ -298,9 +295,6 @@
     <t>Post Retrieval</t>
   </si>
   <si>
-    <t>Type</t>
-  </si>
-  <si>
     <t>Datasets</t>
   </si>
   <si>
@@ -355,9 +349,6 @@
     <t>Chunk Overlap</t>
   </si>
   <si>
-    <t>Hugging Face Embeddings: sentence-transformers/all-mpnet-base-v2</t>
-  </si>
-  <si>
     <t>Qwen 3.5:2b</t>
   </si>
   <si>
@@ -383,13 +374,55 @@
   </si>
   <si>
     <t>Environment</t>
+  </si>
+  <si>
+    <t>Hallucination Metric</t>
+  </si>
+  <si>
+    <t>Answer Relavancy</t>
+  </si>
+  <si>
+    <t>Faithfullness Metric</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>Borderline</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Results</t>
+  </si>
+  <si>
+    <t>Metric</t>
+  </si>
+  <si>
+    <t>sentence-transformers/all-mpnet-base-v2: Hugging Face Embeddings</t>
+  </si>
+  <si>
+    <t>&gt;0.5, &gt;=0</t>
+  </si>
+  <si>
+    <t>&gt;0.5, &gt;=1</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Vector Storage</t>
+  </si>
+  <si>
+    <t>ChromaDB</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -498,8 +531,51 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="26"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF002060"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -556,12 +632,57 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF002060"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="-0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -624,14 +745,175 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thick">
-        <color theme="9"/>
+        <color rgb="FF002060"/>
+      </left>
+      <right/>
+      <top style="thick">
+        <color rgb="FF002060"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color rgb="FF002060"/>
+      </right>
+      <top style="thick">
+        <color rgb="FF002060"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF002060"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color rgb="FF002060"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF002060"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color rgb="FF002060"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color rgb="FF002060"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color rgb="FF002060"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF002060"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF002060"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF002060"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF002060"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF002060"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF002060"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF002060"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF002060"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF002060"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF002060"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF002060"/>
       </left>
       <right style="thick">
-        <color theme="9"/>
+        <color rgb="FF002060"/>
       </right>
       <top style="thick">
-        <color theme="9"/>
+        <color rgb="FF002060"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="slantDashDot">
+        <color rgb="FFFF0000"/>
+      </left>
+      <right style="slantDashDot">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top style="slantDashDot">
+        <color rgb="FFFF0000"/>
       </top>
       <bottom style="thin">
         <color indexed="64"/>
@@ -639,35 +921,94 @@
       <diagonal/>
     </border>
     <border>
+      <left style="slantDashDot">
+        <color rgb="FFFF0000"/>
+      </left>
+      <right style="slantDashDot">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="slantDashDot">
+        <color rgb="FFFF0000"/>
+      </left>
+      <right style="slantDashDot">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="slantDashDot">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thick">
-        <color theme="9"/>
+        <color rgb="FF002060"/>
       </left>
       <right style="thick">
-        <color theme="9"/>
+        <color rgb="FF002060"/>
       </right>
-      <top/>
+      <top style="thin">
+        <color rgb="FF002060"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FF002060"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF002060"/>
+      </left>
+      <right style="thick">
+        <color rgb="FF002060"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF002060"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thick">
-        <color theme="9"/>
+      <left style="thin">
+        <color indexed="64"/>
       </left>
-      <right style="thick">
-        <color theme="9"/>
-      </right>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
       <top/>
-      <bottom style="thick">
-        <color theme="9"/>
+      <bottom style="thin">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -798,55 +1139,153 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="fill" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="16" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="16" xfId="4" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="18" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="5">
+    <cellStyle name="Bad" xfId="3" builtinId="27"/>
+    <cellStyle name="Good" xfId="2" builtinId="26"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Neutral" xfId="4" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF5050"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1781,297 +2220,361 @@
     <col min="14" max="14" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="I3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="9" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D9" s="53" t="s">
+    <row r="3" spans="4:11" ht="33.75" x14ac:dyDescent="0.5">
+      <c r="E3" s="89" t="s">
+        <v>119</v>
+      </c>
+      <c r="F3" s="89"/>
+      <c r="G3" s="89"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="58"/>
+    </row>
+    <row r="8" spans="4:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="9" spans="4:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D9" s="87" t="s">
+        <v>97</v>
+      </c>
+      <c r="E9" s="88"/>
+    </row>
+    <row r="10" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D10" s="53" t="s">
+        <v>102</v>
+      </c>
+      <c r="E10" s="54">
+        <v>1000</v>
+      </c>
+      <c r="G10" s="77" t="s">
+        <v>120</v>
+      </c>
+      <c r="H10" s="78"/>
+    </row>
+    <row r="11" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D11" s="53" t="s">
+        <v>103</v>
+      </c>
+      <c r="E11" s="54">
+        <v>100</v>
+      </c>
+      <c r="G11" s="69" t="s">
+        <v>122</v>
+      </c>
+      <c r="H11" s="71" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="12" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D12" s="53" t="s">
+        <v>98</v>
+      </c>
+      <c r="E12" s="55" t="s">
+        <v>121</v>
+      </c>
+      <c r="G12" s="69">
+        <v>0.5</v>
+      </c>
+      <c r="H12" s="72" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="13" spans="4:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D13" s="53" t="s">
         <v>99</v>
       </c>
-      <c r="E9" s="53"/>
-    </row>
-    <row r="10" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D10" s="44" t="s">
+      <c r="E13" s="54" t="s">
         <v>104</v>
       </c>
-      <c r="E10" s="44">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="11" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D11" s="44" t="s">
+      <c r="G13" s="70" t="s">
+        <v>123</v>
+      </c>
+      <c r="H13" s="73" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="14" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D14" s="53" t="s">
+        <v>100</v>
+      </c>
+      <c r="E14" s="54" t="s">
         <v>105</v>
       </c>
-      <c r="E11" s="44">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="12" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D12" s="44" t="s">
-        <v>100</v>
-      </c>
-      <c r="E12" s="48" t="s">
+    </row>
+    <row r="15" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D15" s="53" t="s">
+        <v>125</v>
+      </c>
+      <c r="E15" s="54" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="16" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D16" s="53" t="s">
+        <v>101</v>
+      </c>
+      <c r="E16" s="54" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="13" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D13" s="44" t="s">
-        <v>101</v>
-      </c>
-      <c r="E13" s="44" t="s">
+    <row r="17" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D17" s="56" t="s">
+        <v>108</v>
+      </c>
+      <c r="E17" s="57" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="14" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D14" s="44" t="s">
-        <v>102</v>
-      </c>
-      <c r="E14" s="44" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="15" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D15" s="44" t="s">
-        <v>103</v>
-      </c>
-      <c r="E15" s="44" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="16" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D16" s="44" t="s">
-        <v>111</v>
-      </c>
-      <c r="E16" s="44" t="s">
-        <v>110</v>
-      </c>
-    </row>
+    <row r="18" spans="3:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="20" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C20" s="45" t="s">
+        <v>79</v>
+      </c>
+      <c r="D20" s="86" t="s">
+        <v>86</v>
+      </c>
+      <c r="E20" s="86"/>
+      <c r="F20" s="81" t="s">
+        <v>84</v>
+      </c>
+      <c r="G20" s="81"/>
+      <c r="H20" s="81"/>
+      <c r="I20" s="81"/>
+      <c r="J20" s="81"/>
+      <c r="K20" s="81"/>
+    </row>
+    <row r="21" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C21" s="74" t="s">
+        <v>83</v>
+      </c>
+      <c r="D21" s="74" t="s">
+        <v>124</v>
+      </c>
+      <c r="E21" s="79" t="s">
         <v>80</v>
       </c>
-      <c r="D20" s="52" t="s">
+      <c r="F21" s="82" t="s">
+        <v>95</v>
+      </c>
+      <c r="G21" s="83"/>
+      <c r="H21" s="83"/>
+      <c r="I21" s="84" t="s">
+        <v>85</v>
+      </c>
+      <c r="J21" s="85"/>
+      <c r="K21" s="85"/>
+    </row>
+    <row r="22" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C22" s="75"/>
+      <c r="D22" s="76"/>
+      <c r="E22" s="80"/>
+      <c r="F22" s="59" t="s">
+        <v>81</v>
+      </c>
+      <c r="G22" s="49" t="s">
+        <v>82</v>
+      </c>
+      <c r="H22" s="50" t="s">
+        <v>96</v>
+      </c>
+      <c r="I22" s="62" t="s">
+        <v>81</v>
+      </c>
+      <c r="J22" s="51" t="s">
+        <v>82</v>
+      </c>
+      <c r="K22" s="52" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="23" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C23" s="75"/>
+      <c r="D23" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="E20" s="52"/>
-      <c r="F20" s="49" t="s">
-        <v>85</v>
-      </c>
-      <c r="G20" s="49"/>
-      <c r="H20" s="49"/>
-      <c r="I20" s="49"/>
-      <c r="J20" s="49"/>
-      <c r="K20" s="49"/>
-    </row>
-    <row r="21" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C21" s="46"/>
-      <c r="D21" s="47" t="s">
+      <c r="E23" s="47" t="s">
         <v>87</v>
       </c>
-      <c r="E21" s="47" t="s">
-        <v>81</v>
-      </c>
-      <c r="F21" s="56" t="s">
-        <v>97</v>
-      </c>
-      <c r="G21" s="50"/>
-      <c r="H21" s="50"/>
-      <c r="I21" s="61" t="s">
-        <v>86</v>
-      </c>
-      <c r="J21" s="51"/>
-      <c r="K21" s="51"/>
-    </row>
-    <row r="22" spans="3:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="C22" s="46"/>
-      <c r="D22" s="46"/>
-      <c r="E22" s="54"/>
-      <c r="F22" s="57" t="s">
-        <v>82</v>
-      </c>
-      <c r="G22" s="55" t="s">
-        <v>83</v>
-      </c>
-      <c r="H22" s="60" t="s">
-        <v>98</v>
-      </c>
-      <c r="I22" s="57" t="s">
-        <v>82</v>
-      </c>
-      <c r="J22" s="55" t="s">
-        <v>83</v>
-      </c>
-      <c r="K22" s="45" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="23" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="D23" s="44" t="s">
+      <c r="F23" s="60">
+        <v>0</v>
+      </c>
+      <c r="G23" s="48">
+        <v>1</v>
+      </c>
+      <c r="H23" s="47">
+        <v>0</v>
+      </c>
+      <c r="I23" s="60">
+        <v>1</v>
+      </c>
+      <c r="J23" s="48">
+        <v>1</v>
+      </c>
+      <c r="K23" s="46">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C24" s="75"/>
+      <c r="D24" s="46" t="s">
         <v>90</v>
       </c>
-      <c r="E23" s="44" t="s">
+      <c r="E24" s="47" t="s">
         <v>89</v>
       </c>
-      <c r="F23" s="58">
+      <c r="F24" s="60">
         <v>0</v>
       </c>
-      <c r="G23" s="44">
+      <c r="G24" s="48">
         <v>1</v>
       </c>
-      <c r="H23" s="44">
+      <c r="H24" s="47">
+        <v>1</v>
+      </c>
+      <c r="I24" s="60">
+        <v>1</v>
+      </c>
+      <c r="J24" s="48">
+        <v>1</v>
+      </c>
+      <c r="K24" s="46">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="25" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C25" s="75"/>
+      <c r="D25" s="46" t="s">
+        <v>92</v>
+      </c>
+      <c r="E25" s="47" t="s">
+        <v>91</v>
+      </c>
+      <c r="F25" s="60">
         <v>0</v>
       </c>
-      <c r="I23" s="58">
+      <c r="G25" s="48">
+        <v>0.75</v>
+      </c>
+      <c r="H25" s="47">
+        <v>0</v>
+      </c>
+      <c r="I25" s="60">
         <v>1</v>
       </c>
-      <c r="J23" s="44">
+      <c r="J25" s="48">
         <v>1</v>
       </c>
-      <c r="K23" s="44">
+      <c r="K25" s="46">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="D24" s="44" t="s">
-        <v>92</v>
-      </c>
-      <c r="E24" s="44" t="s">
-        <v>91</v>
-      </c>
-      <c r="F24" s="58">
+    <row r="26" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C26" s="75"/>
+      <c r="D26" s="46" t="s">
+        <v>112</v>
+      </c>
+      <c r="E26" s="47" t="s">
+        <v>110</v>
+      </c>
+      <c r="F26" s="60">
         <v>0</v>
       </c>
-      <c r="G24" s="44">
+      <c r="G26" s="48">
+        <v>0.84599999999999997</v>
+      </c>
+      <c r="H26" s="47">
         <v>1</v>
       </c>
-      <c r="H24" s="44">
+      <c r="I26" s="60">
         <v>1</v>
       </c>
-      <c r="I24" s="58">
+      <c r="J26" s="48">
         <v>1</v>
       </c>
-      <c r="J24" s="44">
+      <c r="K26" s="46">
         <v>1</v>
       </c>
-      <c r="K24" s="44">
+    </row>
+    <row r="27" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C27" s="75"/>
+      <c r="D27" s="46" t="s">
+        <v>93</v>
+      </c>
+      <c r="E27" s="47" t="s">
+        <v>109</v>
+      </c>
+      <c r="F27" s="60">
+        <v>1</v>
+      </c>
+      <c r="G27" s="48">
+        <v>1</v>
+      </c>
+      <c r="H27" s="47">
+        <v>1</v>
+      </c>
+      <c r="I27" s="60">
+        <v>0</v>
+      </c>
+      <c r="J27" s="48">
+        <v>1</v>
+      </c>
+      <c r="K27" s="46">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C28" s="76"/>
+      <c r="D28" s="46" t="s">
+        <v>94</v>
+      </c>
+      <c r="E28" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="F28" s="61">
+        <v>0</v>
+      </c>
+      <c r="G28" s="48">
+        <v>0.8</v>
+      </c>
+      <c r="H28" s="47">
+        <v>0</v>
+      </c>
+      <c r="I28" s="61">
+        <v>0</v>
+      </c>
+      <c r="J28" s="48">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="25" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C25" s="44" t="s">
-        <v>84</v>
-      </c>
-      <c r="D25" s="44" t="s">
-        <v>94</v>
-      </c>
-      <c r="E25" s="44" t="s">
-        <v>93</v>
-      </c>
-      <c r="F25" s="58">
-        <v>0</v>
-      </c>
-      <c r="G25" s="44">
-        <v>0.75</v>
-      </c>
-      <c r="H25" s="44">
-        <v>0</v>
-      </c>
-      <c r="I25" s="58">
-        <v>1</v>
-      </c>
-      <c r="J25" s="44">
-        <v>1</v>
-      </c>
-      <c r="K25" s="44">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="D26" s="44" t="s">
-        <v>115</v>
-      </c>
-      <c r="E26" s="44" t="s">
-        <v>113</v>
-      </c>
-      <c r="F26" s="58">
-        <v>0</v>
-      </c>
-      <c r="G26" s="44">
-        <v>0.84599999999999997</v>
-      </c>
-      <c r="H26" s="44">
-        <v>1</v>
-      </c>
-      <c r="I26" s="58">
-        <v>1</v>
-      </c>
-      <c r="J26" s="44">
-        <v>1</v>
-      </c>
-      <c r="K26" s="44">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="D27" s="44" t="s">
-        <v>95</v>
-      </c>
-      <c r="E27" s="44" t="s">
-        <v>112</v>
-      </c>
-      <c r="F27" s="58">
-        <v>1</v>
-      </c>
-      <c r="G27" s="44">
-        <v>1</v>
-      </c>
-      <c r="H27" s="44">
-        <v>1</v>
-      </c>
-      <c r="I27" s="58">
-        <v>0</v>
-      </c>
-      <c r="J27" s="44">
-        <v>1</v>
-      </c>
-      <c r="K27" s="44">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="D28" s="44" t="s">
-        <v>96</v>
-      </c>
-      <c r="E28" s="44" t="s">
-        <v>114</v>
-      </c>
-      <c r="F28" s="58">
-        <v>0</v>
-      </c>
-      <c r="G28" s="44">
-        <v>0.8</v>
-      </c>
-      <c r="H28" s="44">
-        <v>0</v>
-      </c>
-      <c r="I28" s="58">
-        <v>0</v>
-      </c>
-      <c r="J28" s="44">
-        <v>0.5</v>
-      </c>
-      <c r="K28" s="44">
+      <c r="K28" s="46">
         <v>0.25</v>
       </c>
     </row>
     <row r="29" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E29" s="44"/>
-      <c r="F29" s="59"/>
-      <c r="I29" s="59"/>
-    </row>
-    <row r="30" spans="3:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    </row>
+    <row r="30" spans="3:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="D30" s="66" t="s">
+        <v>81</v>
+      </c>
+      <c r="E30" s="63" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="31" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="D31" s="68" t="s">
+        <v>82</v>
+      </c>
+      <c r="E31" s="64" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="32" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D32" s="67" t="s">
+        <v>96</v>
+      </c>
+      <c r="E32" s="65" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="33" spans="12:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="36" spans="12:12" x14ac:dyDescent="0.25">
       <c r="L36" s="44"/>
     </row>
@@ -2082,12 +2585,17 @@
       <c r="L38" s="44"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="10">
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="C21:C28"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="E21:E22"/>
     <mergeCell ref="F20:K20"/>
     <mergeCell ref="F21:H21"/>
     <mergeCell ref="I21:K21"/>
     <mergeCell ref="D20:E20"/>
-    <mergeCell ref="D9:E9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added presentation & MPR for month of October
</commit_message>
<xml_diff>
--- a/Records.xlsx
+++ b/Records.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Projects\rag-dissertation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0E3FD74-BA31-4EA2-9074-2AE5C73790FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E801F54A-BE56-4028-B4C4-C712C5283F73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{F211E78F-65A6-4528-B59A-5C2BEDBB7ED5}"/>
   </bookViews>
@@ -403,12 +403,6 @@
     <t>sentence-transformers/all-mpnet-base-v2: Hugging Face Embeddings</t>
   </si>
   <si>
-    <t>&gt;0.5, &gt;=0</t>
-  </si>
-  <si>
-    <t>&gt;0.5, &gt;=1</t>
-  </si>
-  <si>
     <t>Field</t>
   </si>
   <si>
@@ -416,6 +410,12 @@
   </si>
   <si>
     <t>ChromaDB</t>
+  </si>
+  <si>
+    <t>&gt;0.5&gt;=0</t>
+  </si>
+  <si>
+    <t>&lt;0.5 &gt;=1</t>
   </si>
 </sst>
 </file>
@@ -1223,6 +1223,15 @@
     <xf numFmtId="0" fontId="16" fillId="10" borderId="18" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1261,15 +1270,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -2221,21 +2221,21 @@
   </cols>
   <sheetData>
     <row r="3" spans="4:11" ht="33.75" x14ac:dyDescent="0.5">
-      <c r="E3" s="89" t="s">
+      <c r="E3" s="76" t="s">
         <v>119</v>
       </c>
-      <c r="F3" s="89"/>
-      <c r="G3" s="89"/>
+      <c r="F3" s="76"/>
+      <c r="G3" s="76"/>
       <c r="I3" s="58"/>
       <c r="J3" s="58"/>
       <c r="K3" s="58"/>
     </row>
     <row r="8" spans="4:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="9" spans="4:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D9" s="87" t="s">
+      <c r="D9" s="74" t="s">
         <v>97</v>
       </c>
-      <c r="E9" s="88"/>
+      <c r="E9" s="75"/>
     </row>
     <row r="10" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D10" s="53" t="s">
@@ -2244,10 +2244,10 @@
       <c r="E10" s="54">
         <v>1000</v>
       </c>
-      <c r="G10" s="77" t="s">
+      <c r="G10" s="80" t="s">
         <v>120</v>
       </c>
-      <c r="H10" s="78"/>
+      <c r="H10" s="81"/>
     </row>
     <row r="11" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D11" s="53" t="s">
@@ -2257,7 +2257,7 @@
         <v>100</v>
       </c>
       <c r="G11" s="69" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="H11" s="71" t="s">
         <v>116</v>
@@ -2285,7 +2285,7 @@
         <v>104</v>
       </c>
       <c r="G13" s="70" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="H13" s="73" t="s">
         <v>118</v>
@@ -2301,10 +2301,10 @@
     </row>
     <row r="15" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D15" s="53" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E15" s="54" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16" spans="4:11" x14ac:dyDescent="0.25">
@@ -2328,44 +2328,44 @@
       <c r="C20" s="45" t="s">
         <v>79</v>
       </c>
-      <c r="D20" s="86" t="s">
+      <c r="D20" s="89" t="s">
         <v>86</v>
       </c>
-      <c r="E20" s="86"/>
-      <c r="F20" s="81" t="s">
+      <c r="E20" s="89"/>
+      <c r="F20" s="84" t="s">
         <v>84</v>
       </c>
-      <c r="G20" s="81"/>
-      <c r="H20" s="81"/>
-      <c r="I20" s="81"/>
-      <c r="J20" s="81"/>
-      <c r="K20" s="81"/>
+      <c r="G20" s="84"/>
+      <c r="H20" s="84"/>
+      <c r="I20" s="84"/>
+      <c r="J20" s="84"/>
+      <c r="K20" s="84"/>
     </row>
     <row r="21" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C21" s="74" t="s">
+      <c r="C21" s="77" t="s">
         <v>83</v>
       </c>
-      <c r="D21" s="74" t="s">
-        <v>124</v>
-      </c>
-      <c r="E21" s="79" t="s">
+      <c r="D21" s="77" t="s">
+        <v>122</v>
+      </c>
+      <c r="E21" s="82" t="s">
         <v>80</v>
       </c>
-      <c r="F21" s="82" t="s">
+      <c r="F21" s="85" t="s">
         <v>95</v>
       </c>
-      <c r="G21" s="83"/>
-      <c r="H21" s="83"/>
-      <c r="I21" s="84" t="s">
+      <c r="G21" s="86"/>
+      <c r="H21" s="86"/>
+      <c r="I21" s="87" t="s">
         <v>85</v>
       </c>
-      <c r="J21" s="85"/>
-      <c r="K21" s="85"/>
+      <c r="J21" s="88"/>
+      <c r="K21" s="88"/>
     </row>
     <row r="22" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C22" s="75"/>
-      <c r="D22" s="76"/>
-      <c r="E22" s="80"/>
+      <c r="C22" s="78"/>
+      <c r="D22" s="79"/>
+      <c r="E22" s="83"/>
       <c r="F22" s="59" t="s">
         <v>81</v>
       </c>
@@ -2386,7 +2386,7 @@
       </c>
     </row>
     <row r="23" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C23" s="75"/>
+      <c r="C23" s="78"/>
       <c r="D23" s="46" t="s">
         <v>88</v>
       </c>
@@ -2413,7 +2413,7 @@
       </c>
     </row>
     <row r="24" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C24" s="75"/>
+      <c r="C24" s="78"/>
       <c r="D24" s="46" t="s">
         <v>90</v>
       </c>
@@ -2440,7 +2440,7 @@
       </c>
     </row>
     <row r="25" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C25" s="75"/>
+      <c r="C25" s="78"/>
       <c r="D25" s="46" t="s">
         <v>92</v>
       </c>
@@ -2467,7 +2467,7 @@
       </c>
     </row>
     <row r="26" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C26" s="75"/>
+      <c r="C26" s="78"/>
       <c r="D26" s="46" t="s">
         <v>112</v>
       </c>
@@ -2494,7 +2494,7 @@
       </c>
     </row>
     <row r="27" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C27" s="75"/>
+      <c r="C27" s="78"/>
       <c r="D27" s="46" t="s">
         <v>93</v>
       </c>
@@ -2521,7 +2521,7 @@
       </c>
     </row>
     <row r="28" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C28" s="76"/>
+      <c r="C28" s="79"/>
       <c r="D28" s="46" t="s">
         <v>94</v>
       </c>

</xml_diff>